<commit_message>
Step 6.7: Frontend - Import et gestion des mensualités + Step 6.8: Plan multi-crédits avec sous-onglets
- Ajout composants LoanPaymentFileUpload, LoanPaymentPreviewModal, LoanPaymentTable
- Import Excel avec preview et validation
- Tableau avec checkboxes et suppression multiple
- Icônes ✏️ et 🗑️ dans Actions
- Correction validation Pydantic (capital >= 0 au lieu de > 0)
- Ajout Step 6.8 dans plan d'implémentation (multi-crédits avec sous-onglets)
</commit_message>
<xml_diff>
--- a/backend/data/input/trades/mappings_2025-12-25.xlsx
+++ b/backend/data/input/trades/mappings_2025-12-25.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D135"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -421,10 +421,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>PRLV SEPA FREE TELECOM</v>
+        <v>ASSURANCE DU PROPRIETAIRE NON O</v>
       </c>
       <c r="B2" t="str">
-        <v>Livebox</v>
+        <v>assurance PNO</v>
       </c>
       <c r="C2" t="str">
         <v>Charges</v>
@@ -435,41 +435,41 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>VIR SEPA VIREMENT GESTION - LOU</v>
+        <v>COMMIS.PRET</v>
       </c>
       <c r="B3" t="str">
-        <v>Agence loc/menage</v>
+        <v>commission pret</v>
       </c>
       <c r="C3" t="str">
         <v>Charges</v>
       </c>
       <c r="D3" t="str">
-        <v>Daily</v>
+        <v>Achat</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ECH PRET CAP+IN 08922 213949 08</v>
+        <v>DEBLOCAGE PRET 08922 213949 04</v>
       </c>
       <c r="B4" t="str">
-        <v>mensualites du pret</v>
+        <v>pret verse a Louis</v>
       </c>
       <c r="C4" t="str">
-        <v>running costs</v>
+        <v>prêt (inflows)</v>
       </c>
       <c r="D4" t="str">
-        <v>Daily</v>
+        <v>Achat</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PRLV SEPA TOTALENERGIES ELECTRI</v>
+        <v>ECH PRET CAP+IN 08922 213949 04</v>
       </c>
       <c r="B5" t="str">
-        <v>electricite</v>
+        <v>mensualites du pret</v>
       </c>
       <c r="C5" t="str">
-        <v>Charges</v>
+        <v>running costs</v>
       </c>
       <c r="D5" t="str">
         <v>Daily</v>
@@ -477,13 +477,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>VIR AIRBNB PAYMENTS LUXEMBOU</v>
+        <v>ECH PRET INT</v>
       </c>
       <c r="B6" t="str">
-        <v>loyers recu</v>
+        <v>interets mensuelles pret</v>
       </c>
       <c r="C6" t="str">
-        <v>Produit</v>
+        <v>running costs</v>
       </c>
       <c r="D6" t="str">
         <v>Daily</v>
@@ -491,10 +491,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PRLV SEPA SDC 17 GLANDEVES</v>
+        <v>F COTIS EUC.CONFORT</v>
       </c>
       <c r="B7" t="str">
-        <v>charges copro</v>
+        <v>cotisations carte bleu CM</v>
       </c>
       <c r="C7" t="str">
         <v>Charges</v>
@@ -505,10 +505,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>VIR SEPA LOUIS GARNIER ABNB</v>
+        <v>F RETRO EUC.CONFORT</v>
       </c>
       <c r="B8" t="str">
-        <v>Agence loc/menage</v>
+        <v>cotisations carte bleu CM</v>
       </c>
       <c r="C8" t="str">
         <v>Charges</v>
@@ -519,27 +519,27 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>VIR TOTALENERGIES ELECTRICIT</v>
+        <v>PAIEMENT CB 0410 PARIS</v>
       </c>
       <c r="B9" t="str">
-        <v>electricite</v>
+        <v>depenses perso</v>
       </c>
       <c r="C9" t="str">
-        <v>Charges</v>
+        <v>Perso</v>
       </c>
       <c r="D9" t="str">
-        <v>Daily</v>
+        <v>Achat</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>VIR SEPA D.R MACONNERIE</v>
+        <v>PAIEMENT CB 0609 PARIS RODIN</v>
       </c>
       <c r="B10" t="str">
-        <v>travaux</v>
+        <v>depenses perso</v>
       </c>
       <c r="C10" t="str">
-        <v>ammortissements</v>
+        <v>Perso</v>
       </c>
       <c r="D10" t="str">
         <v>Achat</v>
@@ -547,97 +547,97 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>DEBLOCAGE PRET 0892221394908</v>
+        <v>PRLV SEPA DIRECTION GENERALE DE</v>
       </c>
       <c r="B11" t="str">
-        <v>pret verse a Louis travaux</v>
+        <v>taxe fonciere</v>
       </c>
       <c r="C11" t="str">
-        <v>prêt (inflows)</v>
+        <v>Impots</v>
       </c>
       <c r="D11" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>VIR SUITE ERREUR VIREMENT</v>
+        <v>PRLV SEPA DRAGON-MIROIRS</v>
       </c>
       <c r="B12" t="str">
-        <v>travaux</v>
+        <v>charges copro</v>
       </c>
       <c r="C12" t="str">
-        <v>ammortissements</v>
+        <v>Charges</v>
       </c>
       <c r="D12" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>VIR SEPA AMEUBLEA - 20240711-LG</v>
+        <v>PRLV SEPA FREE TELECOM</v>
       </c>
       <c r="B13" t="str">
-        <v>meubles</v>
+        <v>livebox/internet</v>
       </c>
       <c r="C13" t="str">
-        <v>ammortissements</v>
+        <v>Charges</v>
       </c>
       <c r="D13" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>VIR SEPA COMMISSION APPART MARS</v>
+        <v>PRLV SEPA MATMUT CO</v>
       </c>
       <c r="B14" t="str">
-        <v>commission recherche KP</v>
+        <v>assurance PNO</v>
       </c>
       <c r="C14" t="str">
         <v>Charges</v>
       </c>
       <c r="D14" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>COMMISSION KEVIN PAYEN</v>
+        <v>PRLV SEPA MATMUT ROUEN</v>
       </c>
       <c r="B15" t="str">
-        <v>commission remboursement masteos</v>
+        <v>assurance PNO</v>
       </c>
       <c r="C15" t="str">
         <v>Charges</v>
       </c>
       <c r="D15" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>REMBOURSEMENT MASTEOS</v>
+        <v>PRLV SEPA TOTALENERGIES ELECTRI</v>
       </c>
       <c r="B16" t="str">
-        <v>commission remboursement masteos</v>
+        <v>electricite</v>
       </c>
       <c r="C16" t="str">
         <v>Charges</v>
       </c>
       <c r="D16" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>RB.IMP 04/24 0892221394908</v>
+        <v>REF: SUITE SINISTRE DU 03/01/22</v>
       </c>
       <c r="B17" t="str">
-        <v>mensualites du pret</v>
+        <v>Remboursement assurance sinistre 3/01</v>
       </c>
       <c r="C17" t="str">
-        <v>running costs</v>
+        <v>Produit</v>
       </c>
       <c r="D17" t="str">
         <v>Daily</v>
@@ -645,13 +645,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>VIR DE APPARTEMENT EVRY</v>
+        <v>SOUSCRIPTION PART SOCIALE A</v>
       </c>
       <c r="B18" t="str">
-        <v>compte courant</v>
+        <v>souscription part sociale</v>
       </c>
       <c r="C18" t="str">
-        <v>Perso</v>
+        <v>Charges</v>
       </c>
       <c r="D18" t="str">
         <v>Achat</v>
@@ -659,13 +659,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>COMMIS PRET 08922 213949 08</v>
+        <v>VIR INST LGC SASU</v>
       </c>
       <c r="B19" t="str">
-        <v>frais dossier</v>
+        <v>versement perso de louis</v>
       </c>
       <c r="C19" t="str">
-        <v>Charges</v>
+        <v>Perso</v>
       </c>
       <c r="D19" t="str">
         <v>Achat</v>
@@ -673,10 +673,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>APPORT FRAIS DOSSIER</v>
+        <v>VIR INST LOUIS GARNIER</v>
       </c>
       <c r="B20" t="str">
-        <v>compte courant</v>
+        <v>versement perso de louis</v>
       </c>
       <c r="C20" t="str">
         <v>Perso</v>
@@ -687,41 +687,41 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>pret verse a Louis</v>
+        <v>VIR INST MASTEOS</v>
       </c>
       <c r="B21" t="str">
-        <v>pret verse a Louis</v>
+        <v>rembousement masteos Thierry</v>
       </c>
       <c r="C21" t="str">
-        <v>prêt (inflows)</v>
+        <v>Produit</v>
       </c>
       <c r="D21" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>achat appart</v>
+        <v>VIR INST MASTEOS TRANSACTION</v>
       </c>
       <c r="B22" t="str">
-        <v>pret banque - construction</v>
+        <v>loyers recu</v>
       </c>
       <c r="C22" t="str">
-        <v>ammortissements</v>
+        <v>Produit</v>
       </c>
       <c r="D22" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>frais notaire achat</v>
+        <v>VIR M GARNIER LOUIS</v>
       </c>
       <c r="B23" t="str">
-        <v>frais notaire achat</v>
+        <v>versement perso de louis</v>
       </c>
       <c r="C23" t="str">
-        <v>Charges</v>
+        <v>Perso</v>
       </c>
       <c r="D23" t="str">
         <v>Achat</v>
@@ -729,13 +729,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>frais notaire honoraires</v>
+        <v>VIR M LOUIS GARNIER</v>
       </c>
       <c r="B24" t="str">
-        <v>frais notaire honoraires</v>
+        <v>versement perso de louis</v>
       </c>
       <c r="C24" t="str">
-        <v>Charges</v>
+        <v>Perso</v>
       </c>
       <c r="D24" t="str">
         <v>Achat</v>
@@ -743,41 +743,41 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>commision masteos</v>
+        <v>VIR MANGOPAY</v>
       </c>
       <c r="B25" t="str">
-        <v>commission masteos</v>
+        <v>loyers recu</v>
       </c>
       <c r="C25" t="str">
-        <v>Charges</v>
+        <v>Produit</v>
       </c>
       <c r="D25" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>taxe fonciere</v>
+        <v>VIR SEPA A&amp;D PLOMBERIE</v>
       </c>
       <c r="B26" t="str">
-        <v>taxe fonciere</v>
+        <v>travaux</v>
       </c>
       <c r="C26" t="str">
-        <v>Impots</v>
+        <v>ammortissements</v>
       </c>
       <c r="D26" t="str">
-        <v>Daily</v>
+        <v>Achat</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>cash apport achat notaire</v>
+        <v>VIR SEPA ABDEL Toiture</v>
       </c>
       <c r="B27" t="str">
-        <v>versement perso de louis notaire</v>
+        <v>travaux</v>
       </c>
       <c r="C27" t="str">
-        <v>Perso</v>
+        <v>ammortissements</v>
       </c>
       <c r="D27" t="str">
         <v>Achat</v>
@@ -785,24 +785,24 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>honoraire de rédaction</v>
+        <v>VIR SEPA ABDEL TRAVAUX</v>
       </c>
       <c r="B28" t="str">
-        <v>frais notaire honoraires</v>
+        <v>travaux</v>
       </c>
       <c r="C28" t="str">
         <v>Charges</v>
       </c>
       <c r="D28" t="str">
-        <v>Achat</v>
+        <v>Daily</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>droit de paiement sur Etat pour l'enregistrement de la promesse de vente</v>
+        <v>VIR SEPA LOUIS GARNIER - NOTAIR</v>
       </c>
       <c r="B29" t="str">
-        <v>frais notaire taxes</v>
+        <v>frais notaire 1</v>
       </c>
       <c r="C29" t="str">
         <v>Charges</v>
@@ -813,41 +813,41 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>VIR SEPA VIREMENT GESTION</v>
+        <v>VIR SEPA MASTEOS TRAVAUX</v>
       </c>
       <c r="B30" t="str">
-        <v>Agence loc/menage</v>
+        <v>meubles</v>
       </c>
       <c r="C30" t="str">
-        <v>Charges</v>
+        <v>ammortissements</v>
       </c>
       <c r="D30" t="str">
-        <v>Daily</v>
+        <v>Achat</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>VIR SEPA GESTION ABNB - AVRIL -</v>
+        <v>VIR INST MASTEOS INDEMNISATION MARSEILLE LOUIS GARNIER</v>
       </c>
       <c r="B31" t="str">
-        <v>Agence loc/menage</v>
+        <v>rembousement masteos Thierry</v>
       </c>
       <c r="C31" t="str">
-        <v>Charges</v>
+        <v>Perso</v>
       </c>
       <c r="D31" t="str">
-        <v>Daily</v>
+        <v>Achat</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>VIR SEPA GESTION ABNB - AOUT25</v>
+        <v>VIR MANGOPAY B53FF2B9DA624FEBAB9C1A511C2FC89D MASTEOS 6911163C LOYER 1 HOMEGA</v>
       </c>
       <c r="B32" t="str">
-        <v>Agence loc/menage</v>
+        <v>loyers recu</v>
       </c>
       <c r="C32" t="str">
-        <v>Charges</v>
+        <v>Produit</v>
       </c>
       <c r="D32" t="str">
         <v>Daily</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>VIR SEPA GESTION ABNB - JUIL25</v>
+        <v>PRLV SEPA MATMUT CO C 32F960001396875L 0261348A 00 2022121500006630020001638</v>
       </c>
       <c r="B33" t="str">
-        <v>Agence loc/menage</v>
+        <v>assurance PNO</v>
       </c>
       <c r="C33" t="str">
         <v>Charges</v>
@@ -869,10 +869,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>VIR SEPA VIR GESTION AIRBNB JAN</v>
+        <v>PRLV SEPA DRAGON-MIROIRS 2374385 PROV./CHG COURANTE 01/12/20 PROV./CHG COURANTE 01/12/2022</v>
       </c>
       <c r="B34" t="str">
-        <v>Agence loc/menage</v>
+        <v>charges copro</v>
       </c>
       <c r="C34" t="str">
         <v>Charges</v>
@@ -883,13 +883,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>VIR SEPA REPARATION CLIM</v>
+        <v>VIR MANGOPAY 13411C9597694600ACB37A339153C9A4 MASTEOS 6911163C LOYER 1 HOMEGA</v>
       </c>
       <c r="B35" t="str">
-        <v>travaux</v>
+        <v>loyers recu</v>
       </c>
       <c r="C35" t="str">
-        <v>Charges</v>
+        <v>Produit</v>
       </c>
       <c r="D35" t="str">
         <v>Daily</v>
@@ -897,21 +897,1407 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>VIR INST MR VICTOR BRIAND</v>
+        <v>VIR MANGOPAY D64E8E716D144BFD99C45E0C6B9FF431 MASTEOS 6911163C LOYER 1 HOMEGA</v>
       </c>
       <c r="B36" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>VIR MANGOPAY 134FA7DDB6344F75A92575A5AE96F7C1 MASTEOS 6911163C LOYER 1 HOMEGA</v>
+      </c>
+      <c r="B37" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>PRLV SEPA FREE TELECOM FHD 1162270265 FREE HAUTDEBIT 1162270265</v>
+      </c>
+      <c r="B38" t="str">
+        <v>livebox/internet</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>VIR TRANSFERT LIVRET A BLEU</v>
+      </c>
+      <c r="B39" t="str">
+        <v>virement livret A</v>
+      </c>
+      <c r="C39" t="str">
+        <v>perso</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>VIR MATMUT &amp; CO</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Remboursement travaux Matmtu</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>PRLV SEPA SARL BUDIZ</v>
+      </c>
+      <c r="B41" t="str">
+        <v>comptable budiz</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>PRLV SEPA SYNDICAT DRAGON MIROI</v>
+      </c>
+      <c r="B42" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>VIR SEPA DEGAT DES EAUX 2 - LG</v>
+      </c>
+      <c r="B43" t="str">
+        <v>debit travaux</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>VIR SEPA DEGAT DES EAUX 1 - LOU</v>
+      </c>
+      <c r="B44" t="str">
+        <v>debit travaux</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>VIR SEPA SIPHON DEGAT EAUX</v>
+      </c>
+      <c r="B45" t="str">
+        <v>debit travaux</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>VIR 102780892200021394905</v>
+      </c>
+      <c r="B46" t="str">
+        <v>assurance PNO</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>PRLV SEPA MACIF PRODUCTION-MACI</v>
+      </c>
+      <c r="B47" t="str">
+        <v>assurance PNO</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>VIR SEPA COMPTA BUDIZ</v>
+      </c>
+      <c r="B48" t="str">
+        <v>comptable budiz</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>VIR TOTALENERGIES ELECTRICIT</v>
+      </c>
+      <c r="B49" t="str">
+        <v>electricite</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>F DUPLICATA RELEVE DE COMPTE</v>
+      </c>
+      <c r="B50" t="str">
+        <v>prelevements CM</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>VIR COMPTE COURANT</v>
+      </c>
+      <c r="B51" t="str">
         <v>compte courant</v>
       </c>
-      <c r="C36" t="str">
+      <c r="C51" t="str">
         <v>Perso</v>
       </c>
-      <c r="D36" t="str">
-        <v>Achat</v>
+      <c r="D51" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Virement re√ßu du 06/10/2022</v>
+      </c>
+      <c r="B52" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>RETRO F DUPLICATA RELEVE</v>
+      </c>
+      <c r="B53" t="str">
+        <v>prelevements CM</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>lave linge darty (paiment darty)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>meubles</v>
+      </c>
+      <c r="C54" t="str">
+        <v>ammortissements</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>lave linge darty (inflow pr le payer)</v>
+      </c>
+      <c r="B55" t="str">
+        <v>versement perso de louis</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Perso</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Virement re√ßu du 06/10/2022 (piement des charges)</v>
+      </c>
+      <c r="B56" t="str">
+        <v>versement perso de louis</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Perso</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Virement re√ßu du 06/10/2022 (cash pour payer les charges)</v>
+      </c>
+      <c r="B57" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>VIR PRÊT ACHAT APPART (construction)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>pret banque - construction</v>
+      </c>
+      <c r="C58" t="str">
+        <v>ammortissements</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>VIR PRÊT ACHAT APPART (terrain)</v>
+      </c>
+      <c r="B59" t="str">
+        <v>pret banque - terrain</v>
+      </c>
+      <c r="C59" t="str">
+        <v>ammortissements</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>DEBLOCAGE PRET appart</v>
+      </c>
+      <c r="B60" t="str">
+        <v>pret verse a Louis</v>
+      </c>
+      <c r="C60" t="str">
+        <v>prêt (inflows)</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>frais notaire (cash pour payer)</v>
+      </c>
+      <c r="B61" t="str">
+        <v>versement perso de louis</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Perso</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>frais notaire (paiement notaire)</v>
+      </c>
+      <c r="B62" t="str">
+        <v>frais notaire</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>frais prêt</v>
+      </c>
+      <c r="B63" t="str">
+        <v>frais pret</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>taxe fonciere</v>
+      </c>
+      <c r="B64" t="str">
+        <v>taxe fonciere</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Impots</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>charge copro</v>
+      </c>
+      <c r="B65" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>commision masteos</v>
+      </c>
+      <c r="B66" t="str">
+        <v>honoraires masteos</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>VIR DE MANDA</v>
+      </c>
+      <c r="B67" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>VIR MANGOPAY Garantie</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Caution entree</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>VIR STRIPE</v>
+      </c>
+      <c r="B69" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>PRLV SEPA MANDA</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Cautions retours</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Caution</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Caution entree</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>VIR DE MANDA (remb frais recherce)</v>
+      </c>
+      <c r="B72" t="str">
+        <v>recherche locataire (erreur)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="B73" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>detecteur de fumee</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Extra costs</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>diagnostic manda</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Extra costs</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>recherche locataire (erreur)</v>
+      </c>
+      <c r="B76" t="str">
+        <v>recherche locataire (erreur)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>frais manda</v>
+      </c>
+      <c r="B77" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Encaissement charges locatives</v>
+      </c>
+      <c r="B78" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Encaissement loyer hors charges</v>
+      </c>
+      <c r="B79" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Honoraires de gestion fevrier florian</v>
+      </c>
+      <c r="B80" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Honoraires de gestion janvier</v>
+      </c>
+      <c r="B81" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Loyer +charges Florian mars</v>
+      </c>
+      <c r="B82" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Loyer+charges fevrier Matthieu Lebros</v>
+      </c>
+      <c r="B83" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Loyer+charges fevrier nicolas segala</v>
+      </c>
+      <c r="B84" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Loyer+charges mars candice aubertin</v>
+      </c>
+      <c r="B85" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Loyer+charges mars matthieu lebros</v>
+      </c>
+      <c r="B86" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Loyer+charges mars nicolas segala</v>
+      </c>
+      <c r="B87" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>RETRO   F DUPLICATA RELEVE DE C OPE DU   12/11/24. TVA   0,00 %</v>
+      </c>
+      <c r="B88" t="str">
+        <v>remboursement CM</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>VIR INST OUVERTURE COMPTE MATER VH50782SBVZLFJ01</v>
+      </c>
+      <c r="B89" t="str">
+        <v>ouverture compte matera</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>VIR SEPA CAUTION RETOUR FLORIAN</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Caution Sortie</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>VIR SEPA TRAVAUX LOUIS GARNIER</v>
+      </c>
+      <c r="B91" t="str">
+        <v>debit travaux</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>caution Matthieu</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Caution entree</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>caution Matthieu LUX</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Caution entree</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>caution candice</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Caution entree</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>caution nicolas segala</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Caution entree</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>loyer + charges candice fevrier</v>
+      </c>
+      <c r="B96" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>loyer + charges fevrier Florian</v>
+      </c>
+      <c r="B97" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>prelevement matera avril</v>
+      </c>
+      <c r="B98" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>prelevement matera juin</v>
+      </c>
+      <c r="B99" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>prelevement matera mai</v>
+      </c>
+      <c r="B100" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>prelevement matera mars</v>
+      </c>
+      <c r="B101" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>premier charges candice</v>
+      </c>
+      <c r="B102" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>premier charges nicolas segala</v>
+      </c>
+      <c r="B103" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>premier loyer candice</v>
+      </c>
+      <c r="B104" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>premier loyer nicolas segala</v>
+      </c>
+      <c r="B105" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>regul charges Florian</v>
+      </c>
+      <c r="B106" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>remboursement ouverture compte matera</v>
+      </c>
+      <c r="B107" t="str">
+        <v>ouverture compte matera</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Prelevement - MATERA - comptabilite</v>
+      </c>
+      <c r="B108" t="str">
+        <v>comptable budiz</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Prelevement - MATERA - etat des lieux Eddy</v>
+      </c>
+      <c r="B109" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Prelevement - MATERA - redaction document Eddy</v>
+      </c>
+      <c r="B110" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>VIR CICCG F2025-2978</v>
+      </c>
+      <c r="B111" t="str">
+        <v>remboursement inconnu</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>prelevement matera juillet</v>
+      </c>
+      <c r="B112" t="str">
+        <v>honoraires location</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>VIR PRET ACHAT APPART (construction)</v>
+      </c>
+      <c r="B113" t="str">
+        <v>pret banque - construction</v>
+      </c>
+      <c r="C113" t="str">
+        <v>ammortissements</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>VIR PRET ACHAT APPART (terrain)</v>
+      </c>
+      <c r="B114" t="str">
+        <v>pret banque - terrain</v>
+      </c>
+      <c r="C114" t="str">
+        <v>ammortissements</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>VIR SEPA MASTEOS TRAVAUX n</v>
+      </c>
+      <c r="B115" t="str">
+        <v>meubles</v>
+      </c>
+      <c r="C115" t="str">
+        <v>ammortissements</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Virement recu du 06/10/2022 (cash pour payer les charges)</v>
+      </c>
+      <c r="B116" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Virement recu du 06/10/2022 (piement des charges)</v>
+      </c>
+      <c r="B117" t="str">
+        <v>versement perso de louis</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Perso</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Achat</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>VIR STRIPE MANDA-ZNFQWZHWIWS1XCUOVYWOU2QFWHICZ MANDA</v>
+      </c>
+      <c r="B118" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>PRLV SEPA FREE TELECOM FHD-1340738623 FREE HAUTDEBIT 1340738623</v>
+      </c>
+      <c r="B119" t="str">
+        <v>livebox/internet</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>PRLV SEPA SYNDICAT DRAGON MIROI DS241209-IID1850 APPEL PROVISIONS SUR CHARGES 01 122024 12 12</v>
+      </c>
+      <c r="B120" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>PRLV SEPA SYNDICAT DRAGON MIROI DS241209-IID1883 COTISATION FONDS TRAVAUX 01 12 2024 12 12</v>
+      </c>
+      <c r="B121" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>VIR STRIPE MANDA-Y8TW6R89CTZZVWL55C3UY1Z0IKG9W MANDA</v>
+      </c>
+      <c r="B122" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>VIR STRIPE MANDA-4IS1RAH2PUK22Y3WQUCWRQXNG89NF MANDA</v>
+      </c>
+      <c r="B123" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>VIR TOTALENERGIES ELECTRICIT 0111751477-222702554884 VIREMENT TOTALENERGIES ELECTRICITEET GAZ FRANCE-REFERENCE CLIENT 1117</v>
+      </c>
+      <c r="B124" t="str">
+        <v>electricite</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>PRLV SEPA TOTALENERGIES ELECTRI 0111751477-203013044519 PRELEVEMENT TOTALENERGIES ELECTRICITE ET GAZ FRANCE-REFERENCE CLIENT 1</v>
+      </c>
+      <c r="B125" t="str">
+        <v>electricite</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>RETRO F DUPLICATA RELEVE DE C OPE DU 12/11/24  TVA 0 00 %</v>
+      </c>
+      <c r="B126" t="str">
+        <v>prelevements CM</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>PRLV SEPA SYNDICAT DRAGON MIROI DS250108-IID820 COTISATION FONDS TRAVAUX 01 01 2025 1 12</v>
+      </c>
+      <c r="B127" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>PRLV SEPA SYNDICAT DRAGON MIROI DS250108-IID762 APPEL PROVISIONS SUR CHARGES 01 012025 1 12</v>
+      </c>
+      <c r="B128" t="str">
+        <v>charges copro</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>PRLV SEPA FREE TELECOM FHD-1348225502 FREE HAUTDEBIT 1348225502</v>
+      </c>
+      <c r="B129" t="str">
+        <v>livebox/internet</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>VIR STRIPE MANDA-VBIPM9DQNQYH2J01BJU4FVIVG8RDW MANDA</v>
+      </c>
+      <c r="B130" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C130" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Daily</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>PRLV SEPA MANDA (EX FLATLOOKER) STR16NARBPDYRNUE8IQBQRAN9DHYELBR6P MANDA - DEPOT DE GARANTIE FLAVIE BERTRAND</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Cautions retours</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>PRLV SEPA MANDA (EX FLATLOOKER) STR16NARBQ1S3MFTYEQ27RANHPICRNRWQ7 MANDA - DEPOT DE GARANTIE ENZO BARADAT</v>
+      </c>
+      <c r="B132" t="str">
+        <v>Cautions retours</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>PRLV SEPA MANDA (EX FLATLOOKER) STR16NARBPDYZMCK7PRGZRANAG2UPKYXQG MANDA - DEPOT DE GARANTIE RAPHAELLE BREBION</v>
+      </c>
+      <c r="B133" t="str">
+        <v>Cautions retours</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>PRLV SEPA MANDA (EX FLATLOOKER) STR16NARBPDVS4TSRUPJLRANMQBYVO3L1D MANDA - DEPOT DE GARANTIE MARION TREMBLAY</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Cautions retours</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Cautions</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Cautions</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>VIR STRIPE MANDA-IG8LSEBDSLSJUTIC5LQLEZJVCVXQJ MANDA</v>
+      </c>
+      <c r="B135" t="str">
+        <v>loyers recu</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Daily</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D135"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>